<commit_message>
Actualizar rangos de edad del censo de Riobamba
</commit_message>
<xml_diff>
--- a/riobamba-censo-data/shp/plataforma_a.xlsx
+++ b/riobamba-censo-data/shp/plataforma_a.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Datos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Datos'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Datos'!$A$1:$K$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J78"/>
+  <dimension ref="A1:K78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -498,11 +498,12 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -533,25 +534,30 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>edad0_14</t>
+          <t>edad0_4</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>edad15_29</t>
+          <t>edad5_11</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>edad30_44</t>
+          <t>edad12_17</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>edad45_64</t>
+          <t>edad18_29</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>edad30_64</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>edad65mas</t>
         </is>
@@ -581,15 +587,18 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -617,15 +626,18 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -650,18 +662,21 @@
         <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
         <v>2</v>
       </c>
       <c r="J4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -686,18 +701,21 @@
         <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -722,18 +740,21 @@
         <v>7</v>
       </c>
       <c r="F6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -758,18 +779,21 @@
         <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I7" t="n">
         <v>2</v>
       </c>
       <c r="J7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -794,18 +818,21 @@
         <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H8" t="n">
         <v>3</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J8" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -842,6 +869,9 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
         <v>1</v>
       </c>
     </row>
@@ -866,18 +896,21 @@
         <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -902,18 +935,21 @@
         <v>7</v>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J11" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -941,7 +977,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -950,6 +986,9 @@
         <v>1</v>
       </c>
       <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -974,18 +1013,21 @@
         <v>24</v>
       </c>
       <c r="F13" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="G13" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H13" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I13" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J13" t="n">
+        <v>13</v>
+      </c>
+      <c r="K13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1010,18 +1052,21 @@
         <v>21</v>
       </c>
       <c r="F14" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H14" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I14" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J14" t="n">
+        <v>18</v>
+      </c>
+      <c r="K14" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1046,18 +1091,21 @@
         <v>13</v>
       </c>
       <c r="F15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
         <v>12</v>
       </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>8</v>
       </c>
-      <c r="J15" t="n">
+      <c r="K15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1082,18 +1130,21 @@
         <v>14</v>
       </c>
       <c r="F16" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H16" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J16" t="n">
+        <v>9</v>
+      </c>
+      <c r="K16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1118,18 +1169,21 @@
         <v>4</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1154,18 +1208,21 @@
         <v>6</v>
       </c>
       <c r="F18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I18" t="n">
         <v>2</v>
       </c>
       <c r="J18" t="n">
+        <v>5</v>
+      </c>
+      <c r="K18" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1190,18 +1247,21 @@
         <v>13</v>
       </c>
       <c r="F19" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
+        <v>4</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
         <v>9</v>
       </c>
-      <c r="H19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" t="n">
-        <v>4</v>
-      </c>
       <c r="J19" t="n">
+        <v>5</v>
+      </c>
+      <c r="K19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1226,18 +1286,21 @@
         <v>16</v>
       </c>
       <c r="F20" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I20" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J20" t="n">
+        <v>11</v>
+      </c>
+      <c r="K20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1262,18 +1325,21 @@
         <v>8</v>
       </c>
       <c r="F21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="n">
         <v>6</v>
       </c>
-      <c r="G21" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" t="n">
-        <v>5</v>
-      </c>
-      <c r="I21" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" t="n">
+      <c r="K21" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1298,18 +1364,21 @@
         <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G22" t="n">
         <v>1</v>
       </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
+        <v>2</v>
+      </c>
+      <c r="K22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1337,15 +1406,18 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1370,18 +1442,21 @@
         <v>9</v>
       </c>
       <c r="F24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J24" t="n">
+        <v>6</v>
+      </c>
+      <c r="K24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1406,18 +1481,21 @@
         <v>15</v>
       </c>
       <c r="F25" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" t="n">
+        <v>3</v>
+      </c>
+      <c r="H25" t="n">
+        <v>5</v>
+      </c>
+      <c r="I25" t="n">
+        <v>4</v>
+      </c>
+      <c r="J25" t="n">
         <v>8</v>
       </c>
-      <c r="G25" t="n">
-        <v>6</v>
-      </c>
-      <c r="H25" t="n">
-        <v>7</v>
-      </c>
-      <c r="I25" t="n">
-        <v>1</v>
-      </c>
-      <c r="J25" t="n">
+      <c r="K25" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1442,18 +1520,21 @@
         <v>14</v>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H26" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J26" t="n">
+        <v>12</v>
+      </c>
+      <c r="K26" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1478,18 +1559,21 @@
         <v>11</v>
       </c>
       <c r="F27" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
         <v>6</v>
       </c>
       <c r="H27" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J27" t="n">
+        <v>7</v>
+      </c>
+      <c r="K27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1514,18 +1598,21 @@
         <v>14</v>
       </c>
       <c r="F28" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J28" t="n">
+        <v>5</v>
+      </c>
+      <c r="K28" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1550,18 +1637,21 @@
         <v>7</v>
       </c>
       <c r="F29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I29" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J29" t="n">
+        <v>4</v>
+      </c>
+      <c r="K29" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1586,18 +1676,21 @@
         <v>8</v>
       </c>
       <c r="F30" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G30" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H30" t="n">
+        <v>4</v>
+      </c>
+      <c r="I30" t="n">
+        <v>2</v>
+      </c>
+      <c r="J30" t="n">
         <v>8</v>
       </c>
-      <c r="I30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" t="n">
+      <c r="K30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1622,18 +1715,21 @@
         <v>12</v>
       </c>
       <c r="F31" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H31" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I31" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J31" t="n">
+        <v>8</v>
+      </c>
+      <c r="K31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1658,18 +1754,21 @@
         <v>8</v>
       </c>
       <c r="F32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
         <v>1</v>
       </c>
       <c r="H32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K32" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1694,18 +1793,21 @@
         <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="J33" t="n">
+        <v>3</v>
+      </c>
+      <c r="K33" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1730,18 +1832,21 @@
         <v>10</v>
       </c>
       <c r="F34" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" t="n">
         <v>7</v>
       </c>
-      <c r="H34" t="n">
-        <v>4</v>
-      </c>
-      <c r="I34" t="n">
-        <v>2</v>
-      </c>
       <c r="J34" t="n">
+        <v>6</v>
+      </c>
+      <c r="K34" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1766,18 +1871,21 @@
         <v>9</v>
       </c>
       <c r="F35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G35" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J35" t="n">
+        <v>3</v>
+      </c>
+      <c r="K35" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1802,18 +1910,21 @@
         <v>13</v>
       </c>
       <c r="F36" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36" t="n">
+        <v>8</v>
+      </c>
+      <c r="K36" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1838,18 +1949,21 @@
         <v>14</v>
       </c>
       <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" t="n">
+        <v>2</v>
+      </c>
+      <c r="I37" t="n">
         <v>6</v>
       </c>
-      <c r="G37" t="n">
-        <v>6</v>
-      </c>
-      <c r="H37" t="n">
-        <v>4</v>
-      </c>
-      <c r="I37" t="n">
-        <v>5</v>
-      </c>
       <c r="J37" t="n">
+        <v>9</v>
+      </c>
+      <c r="K37" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1874,18 +1988,21 @@
         <v>4</v>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G38" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I38" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J38" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1913,15 +2030,18 @@
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J39" t="n">
+        <v>5</v>
+      </c>
+      <c r="K39" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1946,18 +2066,21 @@
         <v>7</v>
       </c>
       <c r="F40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G40" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
         <v>2</v>
       </c>
       <c r="I40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J40" t="n">
+        <v>7</v>
+      </c>
+      <c r="K40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1982,18 +2105,21 @@
         <v>6</v>
       </c>
       <c r="F41" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G41" t="n">
+        <v>3</v>
+      </c>
+      <c r="H41" t="n">
+        <v>2</v>
+      </c>
+      <c r="I41" t="n">
         <v>6</v>
       </c>
-      <c r="H41" t="n">
-        <v>3</v>
-      </c>
-      <c r="I41" t="n">
-        <v>3</v>
-      </c>
       <c r="J41" t="n">
+        <v>6</v>
+      </c>
+      <c r="K41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2018,20 +2144,23 @@
         <v>12</v>
       </c>
       <c r="F42" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G42" t="n">
+        <v>2</v>
+      </c>
+      <c r="H42" t="n">
+        <v>2</v>
+      </c>
+      <c r="I42" t="n">
         <v>6</v>
-      </c>
-      <c r="H42" t="n">
-        <v>3</v>
-      </c>
-      <c r="I42" t="n">
-        <v>3</v>
       </c>
       <c r="J42" t="n">
         <v>6</v>
       </c>
+      <c r="K42" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2057,15 +2186,18 @@
         <v>0</v>
       </c>
       <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
         <v>7</v>
       </c>
-      <c r="H43" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" t="n">
-        <v>5</v>
-      </c>
       <c r="J43" t="n">
+        <v>5</v>
+      </c>
+      <c r="K43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2090,18 +2222,21 @@
         <v>17</v>
       </c>
       <c r="F44" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G44" t="n">
         <v>6</v>
       </c>
       <c r="H44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I44" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J44" t="n">
+        <v>11</v>
+      </c>
+      <c r="K44" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2126,18 +2261,21 @@
         <v>6</v>
       </c>
       <c r="F45" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I45" t="n">
         <v>3</v>
       </c>
       <c r="J45" t="n">
+        <v>6</v>
+      </c>
+      <c r="K45" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2165,15 +2303,18 @@
         <v>2</v>
       </c>
       <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1</v>
+      </c>
+      <c r="I46" t="n">
+        <v>7</v>
+      </c>
+      <c r="J46" t="n">
         <v>8</v>
       </c>
-      <c r="H46" t="n">
-        <v>5</v>
-      </c>
-      <c r="I46" t="n">
-        <v>3</v>
-      </c>
-      <c r="J46" t="n">
+      <c r="K46" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2198,18 +2339,21 @@
         <v>13</v>
       </c>
       <c r="F47" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H47" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I47" t="n">
         <v>3</v>
       </c>
       <c r="J47" t="n">
+        <v>9</v>
+      </c>
+      <c r="K47" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2234,18 +2378,21 @@
         <v>8</v>
       </c>
       <c r="F48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G48" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
         <v>6</v>
       </c>
-      <c r="H48" t="n">
-        <v>1</v>
-      </c>
-      <c r="I48" t="n">
-        <v>2</v>
-      </c>
       <c r="J48" t="n">
+        <v>3</v>
+      </c>
+      <c r="K48" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2270,18 +2417,21 @@
         <v>4</v>
       </c>
       <c r="F49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G49" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H49" t="n">
         <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J49" t="n">
+        <v>3</v>
+      </c>
+      <c r="K49" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2306,18 +2456,21 @@
         <v>34</v>
       </c>
       <c r="F50" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="G50" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="H50" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I50" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="J50" t="n">
+        <v>20</v>
+      </c>
+      <c r="K50" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2342,18 +2495,21 @@
         <v>18</v>
       </c>
       <c r="F51" t="n">
+        <v>3</v>
+      </c>
+      <c r="G51" t="n">
+        <v>6</v>
+      </c>
+      <c r="H51" t="n">
+        <v>3</v>
+      </c>
+      <c r="I51" t="n">
         <v>11</v>
       </c>
-      <c r="G51" t="n">
+      <c r="J51" t="n">
         <v>12</v>
       </c>
-      <c r="H51" t="n">
-        <v>7</v>
-      </c>
-      <c r="I51" t="n">
-        <v>5</v>
-      </c>
-      <c r="J51" t="n">
+      <c r="K51" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2378,18 +2534,21 @@
         <v>18</v>
       </c>
       <c r="F52" t="n">
+        <v>3</v>
+      </c>
+      <c r="G52" t="n">
+        <v>5</v>
+      </c>
+      <c r="H52" t="n">
+        <v>3</v>
+      </c>
+      <c r="I52" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" t="n">
         <v>11</v>
       </c>
-      <c r="G52" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" t="n">
-        <v>8</v>
-      </c>
-      <c r="I52" t="n">
-        <v>3</v>
-      </c>
-      <c r="J52" t="n">
+      <c r="K52" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2414,18 +2573,21 @@
         <v>14</v>
       </c>
       <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>2</v>
+      </c>
+      <c r="H53" t="n">
         <v>6</v>
       </c>
-      <c r="G53" t="n">
-        <v>4</v>
-      </c>
-      <c r="H53" t="n">
-        <v>5</v>
-      </c>
       <c r="I53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J53" t="n">
+        <v>6</v>
+      </c>
+      <c r="K53" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2450,18 +2612,21 @@
         <v>32</v>
       </c>
       <c r="F54" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G54" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="H54" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I54" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J54" t="n">
+        <v>23</v>
+      </c>
+      <c r="K54" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2486,18 +2651,21 @@
         <v>13</v>
       </c>
       <c r="F55" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G55" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H55" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I55" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J55" t="n">
+        <v>9</v>
+      </c>
+      <c r="K55" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2522,18 +2690,21 @@
         <v>9</v>
       </c>
       <c r="F56" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G56" t="n">
         <v>4</v>
       </c>
       <c r="H56" t="n">
+        <v>3</v>
+      </c>
+      <c r="I56" t="n">
+        <v>3</v>
+      </c>
+      <c r="J56" t="n">
         <v>7</v>
       </c>
-      <c r="I56" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" t="n">
+      <c r="K56" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2558,18 +2729,21 @@
         <v>9</v>
       </c>
       <c r="F57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J57" t="n">
+        <v>5</v>
+      </c>
+      <c r="K57" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2594,18 +2768,21 @@
         <v>4</v>
       </c>
       <c r="F58" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G58" t="n">
         <v>2</v>
       </c>
       <c r="H58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I58" t="n">
         <v>2</v>
       </c>
       <c r="J58" t="n">
+        <v>4</v>
+      </c>
+      <c r="K58" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2630,18 +2807,21 @@
         <v>2</v>
       </c>
       <c r="F59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H59" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J59" t="n">
+        <v>4</v>
+      </c>
+      <c r="K59" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2666,18 +2846,21 @@
         <v>16</v>
       </c>
       <c r="F60" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G60" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H60" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I60" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J60" t="n">
+        <v>8</v>
+      </c>
+      <c r="K60" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2702,18 +2885,21 @@
         <v>3</v>
       </c>
       <c r="F61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H61" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I61" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J61" t="n">
+        <v>6</v>
+      </c>
+      <c r="K61" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2738,18 +2924,21 @@
         <v>4</v>
       </c>
       <c r="F62" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G62" t="n">
         <v>1</v>
       </c>
       <c r="H62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I62" t="n">
         <v>1</v>
       </c>
       <c r="J62" t="n">
+        <v>3</v>
+      </c>
+      <c r="K62" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2774,18 +2963,21 @@
         <v>13</v>
       </c>
       <c r="F63" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G63" t="n">
         <v>6</v>
       </c>
       <c r="H63" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I63" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J63" t="n">
+        <v>8</v>
+      </c>
+      <c r="K63" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2810,18 +3002,21 @@
         <v>17</v>
       </c>
       <c r="F64" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G64" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H64" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I64" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J64" t="n">
+        <v>11</v>
+      </c>
+      <c r="K64" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2846,18 +3041,21 @@
         <v>4</v>
       </c>
       <c r="F65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G65" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I65" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J65" t="n">
+        <v>2</v>
+      </c>
+      <c r="K65" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2882,18 +3080,21 @@
         <v>12</v>
       </c>
       <c r="F66" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H66" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J66" t="n">
+        <v>10</v>
+      </c>
+      <c r="K66" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2918,18 +3119,21 @@
         <v>13</v>
       </c>
       <c r="F67" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G67" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I67" t="n">
         <v>8</v>
       </c>
       <c r="J67" t="n">
+        <v>10</v>
+      </c>
+      <c r="K67" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2954,10 +3158,10 @@
         <v>6</v>
       </c>
       <c r="F68" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G68" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H68" t="n">
         <v>3</v>
@@ -2966,6 +3170,9 @@
         <v>2</v>
       </c>
       <c r="J68" t="n">
+        <v>5</v>
+      </c>
+      <c r="K68" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2990,18 +3197,21 @@
         <v>11</v>
       </c>
       <c r="F69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G69" t="n">
+        <v>1</v>
+      </c>
+      <c r="H69" t="n">
+        <v>4</v>
+      </c>
+      <c r="I69" t="n">
+        <v>4</v>
+      </c>
+      <c r="J69" t="n">
         <v>7</v>
       </c>
-      <c r="H69" t="n">
-        <v>5</v>
-      </c>
-      <c r="I69" t="n">
-        <v>2</v>
-      </c>
-      <c r="J69" t="n">
+      <c r="K69" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3026,18 +3236,21 @@
         <v>9</v>
       </c>
       <c r="F70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G70" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H70" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J70" t="n">
+        <v>9</v>
+      </c>
+      <c r="K70" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3062,18 +3275,21 @@
         <v>8</v>
       </c>
       <c r="F71" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G71" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H71" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I71" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J71" t="n">
+        <v>8</v>
+      </c>
+      <c r="K71" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3098,18 +3314,21 @@
         <v>34</v>
       </c>
       <c r="F72" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="G72" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H72" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I72" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="J72" t="n">
+        <v>23</v>
+      </c>
+      <c r="K72" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3134,18 +3353,21 @@
         <v>23</v>
       </c>
       <c r="F73" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="G73" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H73" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I73" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J73" t="n">
+        <v>18</v>
+      </c>
+      <c r="K73" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3170,18 +3392,21 @@
         <v>11</v>
       </c>
       <c r="F74" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H74" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J74" t="n">
+        <v>8</v>
+      </c>
+      <c r="K74" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3206,18 +3431,21 @@
         <v>13</v>
       </c>
       <c r="F75" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G75" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H75" t="n">
         <v>1</v>
       </c>
       <c r="I75" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J75" t="n">
+        <v>8</v>
+      </c>
+      <c r="K75" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3242,18 +3470,21 @@
         <v>19</v>
       </c>
       <c r="F76" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G76" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="H76" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I76" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J76" t="n">
+        <v>18</v>
+      </c>
+      <c r="K76" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3278,18 +3509,21 @@
         <v>24</v>
       </c>
       <c r="F77" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="G77" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H77" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I77" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="J77" t="n">
+        <v>16</v>
+      </c>
+      <c r="K77" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3314,23 +3548,26 @@
         <v>22</v>
       </c>
       <c r="F78" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G78" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H78" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I78" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="J78" t="n">
+        <v>17</v>
+      </c>
+      <c r="K78" t="n">
         <v>6</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>